<commit_message>
Example analysis file added
</commit_message>
<xml_diff>
--- a/docs/access-measurement.xlsx
+++ b/docs/access-measurement.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldbankgroup-my.sharepoint.com/personal/dmatekenya_worldbankgroup_org/Documents/Health-Access-Metrics/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mmastro\World_Bank\Health-Access-Metrics\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="162" documentId="8_{697F7D00-295A-BD4C-8F06-CDC7321454BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BE0BFF4-DDF5-D04A-BA8E-585FA81DDCB9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA43EA44-D35A-4DBE-8272-6446C4CE89A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{DB3AFE75-F2D6-4F44-8B50-2FA238768FB1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DB3AFE75-F2D6-4F44-8B50-2FA238768FB1}"/>
   </bookViews>
   <sheets>
     <sheet name="indicators" sheetId="1" r:id="rId1"/>
@@ -40,6 +40,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={28766BF6-05A0-F94D-9920-1D62A8CFFF09}</author>
+    <author>tc={5AF9CD5E-125F-4B84-948E-85D4556279D1}</author>
   </authors>
   <commentList>
     <comment ref="D1" authorId="0" shapeId="0" xr:uid="{28766BF6-05A0-F94D-9920-1D62A8CFFF09}">
@@ -47,7 +48,19 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    The health facility (HF) can be refined to be any, primary, secondary or referral. Furthermore, we can add available care. For example, a HF with at least 50 beds or something like that.</t>
+    The health facility (HF) can be refined to be any, primary, secondary or referral. Furthermore, we can add available care. For example, a HF with at least 50 beds or something like that.
+Reply:
+    It could also be relevant to consider available care in the sense of hospitalization service for a health facility (eg newborn care)</t>
+      </text>
+    </comment>
+    <comment ref="D8" authorId="1" shapeId="0" xr:uid="{5AF9CD5E-125F-4B84-948E-85D4556279D1}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Pregnancy better describe the share and distribution of population at risk.
+Source: https://bmcmedicine.biomedcentral.com/articles/10.1186/s12916-020-01707-6,
+https://doi.org/10.1136/bmjgh-2018-000778. </t>
       </text>
     </comment>
   </commentList>
@@ -55,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="55">
   <si>
     <t>Id</t>
   </si>
@@ -109,6 +122,129 @@
   </si>
   <si>
     <t xml:space="preserve">Population share </t>
+  </si>
+  <si>
+    <t>Number of people</t>
+  </si>
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required Attributes </t>
+  </si>
+  <si>
+    <t>Other Attributes</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>Health facilities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This represents the supply-location of health infrastracture </t>
+  </si>
+  <si>
+    <t>Location (e.g., lat, lon)</t>
+  </si>
+  <si>
+    <t>Type of health facility (e.g, referral, primary etc), number of beds</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>https://data.humdata.org/dataset/hotosm_mwi_health_facilities?force_layout=desktop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Population </t>
+  </si>
+  <si>
+    <t>This represents the clients/demand</t>
+  </si>
+  <si>
+    <t>Location (e.g., gridded population)</t>
+  </si>
+  <si>
+    <t>Time (e.g., census year)</t>
+  </si>
+  <si>
+    <t>https://hub.worldpop.org/geodata/summary?id=49647</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Road netwrok </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infrastructure required to travel </t>
+  </si>
+  <si>
+    <t>Type/class of road and/or speed attributes on road trunks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Road condition </t>
+  </si>
+  <si>
+    <t>No if travel friction surface is available, otherwise yes</t>
+  </si>
+  <si>
+    <t>https://developers.google.com/earth-engine/datasets/catalog/Oxford_MAP_friction_surface_2019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terrain </t>
+  </si>
+  <si>
+    <t>Geographic terrain of the country/region</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel Friction surface </t>
+  </si>
+  <si>
+    <t>Raster layer with modelled travel time using road network and other layers</t>
+  </si>
+  <si>
+    <t>Share of health facilities with direct access to an all-season road</t>
+  </si>
+  <si>
+    <t>Number of HF</t>
+  </si>
+  <si>
+    <t>HF share</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Share of population within  </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>n minutes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  of driving to the nearest referral hospotal</t>
+    </r>
   </si>
   <si>
     <r>
@@ -131,24 +267,23 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>of a health facility</t>
+      <t>of driving to the nearest health facility</t>
     </r>
   </si>
   <si>
-    <t>Number of people</t>
-  </si>
-  <si>
     <r>
-      <t xml:space="preserve">Share of population within  </t>
+      <t xml:space="preserve">Share of health facilities within </t>
     </r>
     <r>
       <rPr>
         <i/>
         <sz val="12"/>
         <color rgb="FFFF0000"/>
-        <rFont val="Calibri (Body)"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </rPr>
-      <t>n minutes</t>
+      <t>n kilometers</t>
     </r>
     <r>
       <rPr>
@@ -158,102 +293,18 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">  of a referral hospotal</t>
+      <t xml:space="preserve"> of an all-season road</t>
     </r>
   </si>
   <si>
-    <t>Dataset</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Required Attributes </t>
-  </si>
-  <si>
-    <t>Other Attributes</t>
-  </si>
-  <si>
-    <t>Required</t>
-  </si>
-  <si>
-    <t>Example</t>
-  </si>
-  <si>
-    <t>Health facilities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">This represents the supply-location of health infrastracture </t>
-  </si>
-  <si>
-    <t>Location (e.g., lat, lon)</t>
-  </si>
-  <si>
-    <t>Type of health facility (e.g, referral, primary etc), number of beds</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>https://data.humdata.org/dataset/hotosm_mwi_health_facilities?force_layout=desktop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Population </t>
-  </si>
-  <si>
-    <t>This represents the clients/demand</t>
-  </si>
-  <si>
-    <t>Location (e.g., gridded population)</t>
-  </si>
-  <si>
-    <t>Time (e.g., census year)</t>
-  </si>
-  <si>
-    <t>https://hub.worldpop.org/geodata/summary?id=49647</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Road netwrok </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Infrastructure required to travel </t>
-  </si>
-  <si>
-    <t>Type/class of road and/or speed attributes on road trunks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Road condition </t>
-  </si>
-  <si>
-    <t>No if travel friction surface is available, otherwise yes</t>
-  </si>
-  <si>
-    <t>https://developers.google.com/earth-engine/datasets/catalog/Oxford_MAP_friction_surface_2019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terrain </t>
-  </si>
-  <si>
-    <t>Geographic terrain of the country/region</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Travel Friction surface </t>
-  </si>
-  <si>
-    <t>Raster layer with modelled travel time using road network and other layers</t>
+    <t>Share of pregnancies located within 2 h to the nearest referral hospital</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -289,6 +340,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -311,10 +376,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -335,6 +416,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="MASTROPIERRO MATTEO" id="{D13CD821-E99A-4FC5-A290-BEEF18C1E465}" userId="S::956554@stud.unive.it::124a7685-118e-43c2-a408-84ed749c8a92" providerId="AD"/>
   <person displayName="Dunstan Matekenya" id="{57F3694D-415C-6548-9D73-12194FDF5305}" userId="S::dmatekenya@worldbankgroup.org::3c2558b3-3bb6-4e66-afbb-69d820939dbc" providerId="AD"/>
 </personList>
 </file>
@@ -639,21 +721,37 @@
   <threadedComment ref="D1" dT="2023-08-19T15:51:28.99" personId="{57F3694D-415C-6548-9D73-12194FDF5305}" id="{28766BF6-05A0-F94D-9920-1D62A8CFFF09}">
     <text>The health facility (HF) can be refined to be any, primary, secondary or referral. Furthermore, we can add available care. For example, a HF with at least 50 beds or something like that.</text>
   </threadedComment>
+  <threadedComment ref="D1" dT="2023-11-01T14:16:53.44" personId="{D13CD821-E99A-4FC5-A290-BEEF18C1E465}" id="{02460AB0-4A0C-4009-B1E8-123DA5A30C63}" parentId="{28766BF6-05A0-F94D-9920-1D62A8CFFF09}">
+    <text>It could also be relevant to consider available care in the sense of hospitalization service for a health facility (eg newborn care)</text>
+  </threadedComment>
+  <threadedComment ref="D8" dT="2023-11-01T14:17:50.85" personId="{D13CD821-E99A-4FC5-A290-BEEF18C1E465}" id="{5AF9CD5E-125F-4B84-948E-85D4556279D1}">
+    <text xml:space="preserve">Pregnancy better describe the share and distribution of population at risk.
+Source: https://bmcmedicine.biomedcentral.com/articles/10.1186/s12916-020-01707-6,
+https://doi.org/10.1136/bmjgh-2018-000778. </text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>2078624491</xltc2:checksum>
+        <xltc2:hyperlink startIndex="84" length="73" url="https://bmcmedicine.biomedcentral.com/articles/10.1186/s12916-020-01707-6"/>
+        <xltc2:hyperlink startIndex="159" length="41" url="https://doi.org/10.1136/bmjgh-2018-000778"/>
+      </x:ext>
+    </extLst>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD229EB8-6437-314E-8ACF-469AD44CA6DF}">
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="6.6640625" customWidth="1"/>
+    <col min="1" max="1" width="6.625" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" customWidth="1"/>
-    <col min="4" max="4" width="58" customWidth="1"/>
+    <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="67.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -663,7 +761,7 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -673,7 +771,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" s="1" customFormat="1">
       <c r="A2">
         <v>1</v>
       </c>
@@ -683,7 +781,7 @@
       <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E2" t="s">
@@ -693,7 +791,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>2</v>
       </c>
@@ -703,7 +801,7 @@
       <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E3" t="s">
@@ -713,7 +811,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>3</v>
       </c>
@@ -723,7 +821,7 @@
       <c r="C4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E4" t="s">
@@ -733,7 +831,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>4</v>
       </c>
@@ -743,7 +841,7 @@
       <c r="C5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E5" t="s">
@@ -753,7 +851,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>5</v>
       </c>
@@ -763,17 +861,17 @@
       <c r="C6" t="s">
         <v>7</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" t="s">
         <v>18</v>
-      </c>
-      <c r="E6" t="s">
-        <v>19</v>
       </c>
       <c r="F6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>6</v>
       </c>
@@ -783,13 +881,73 @@
       <c r="C7" t="s">
         <v>11</v>
       </c>
-      <c r="D7" t="s">
-        <v>20</v>
+      <c r="D7" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="E7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" t="s">
         <v>10</v>
       </c>
     </row>
@@ -803,132 +961,134 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22140040-E112-EB4A-9E79-C4CDC27EA9ED}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="21.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.5" customWidth="1"/>
-    <col min="3" max="3" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.33203125" customWidth="1"/>
+    <col min="1" max="1" width="21.125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.5" style="7" customWidth="1"/>
+    <col min="3" max="3" width="29.625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.5" style="7" customWidth="1"/>
+    <col min="5" max="5" width="18.5" style="7" customWidth="1"/>
+    <col min="6" max="16384" width="11" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" s="4" customFormat="1">
+      <c r="A1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:6" ht="47.25">
+      <c r="A2" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="B2" s="7" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="C2" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="E2" t="s">
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F2" t="s">
+      <c r="B3" s="7" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="C3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="4" spans="1:6" ht="47.25">
+      <c r="A4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="B4" s="7" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="C4" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="31.5">
+      <c r="A6" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>41</v>
-      </c>
-      <c r="E4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" t="s">
-        <v>46</v>
-      </c>
-      <c r="D6" t="s">
-        <v>46</v>
-      </c>
-      <c r="E6" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F3" r:id="rId1" xr:uid="{FC596D91-AC7C-9B4B-9422-74F59E677454}"/>
-    <hyperlink ref="F4" r:id="rId2" xr:uid="{AF7A970C-0963-5D45-A654-CA813B35E04E}"/>
+    <hyperlink ref="F6" r:id="rId2" xr:uid="{AF7A970C-0963-5D45-A654-CA813B35E04E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>